<commit_message>
feat: update bot M5 & M15 to v3.4 (Technical Confluence Suite, Descending Triangle, Anti-Falling Knife, Symmetric RRR, Loop Shield resilience)
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_Terbaru_SMC.xlsx
+++ b/Laporan_Forward_Testing_Model_Terbaru_SMC.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -487,7 +487,7 @@
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="27" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="33" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -642,7 +642,7 @@
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>LightGBM SMC/ICT</t>
+          <t>LightGBM M15 v3.4 (Confluence)</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="Q3" s="4" t="inlineStr">
         <is>
-          <t>LightGBM SMC/ICT</t>
+          <t>LightGBM M15 v3.4 (Confluence)</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="Q4" s="4" t="inlineStr">
         <is>
-          <t>LightGBM SMC/ICT</t>
+          <t>LightGBM M15 v3.4 (Confluence)</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
-          <t>LightGBM SMC/ICT</t>
+          <t>LightGBM M15 v3.4 (Confluence)</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,214 @@
       </c>
       <c r="Q6" s="4" t="inlineStr">
         <is>
-          <t>LightGBM SMC/ICT</t>
+          <t>LightGBM M15 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>2528352257</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10 21:44:55</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10 22:02:27</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>17m 32d</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>4356.418</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>4367.036</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>4341.536</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>4354.983</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M15 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>2529630852</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 01:44:54</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 01:52:03</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>7m 9d</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>4334.166999999999</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>4329.411</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>4340.211</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>4335.417</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M15 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2530715929</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 08:14:55</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 08:16:18</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>1m 23d</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>4333.135</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>4336.135</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>4328.635</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>4336.135</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>-30</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>-3</v>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M15 v3.4 (Confluence)</t>
         </is>
       </c>
     </row>
@@ -937,7 +1144,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -960,7 +1167,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>LightGBM SMC/ICT (28 Fitur SMC/ICT + DXY + MTF)</t>
+          <t>LightGBM M15 v3.4 (Confluence) (28 Fitur SMC/ICT + DXY + MTF)</t>
         </is>
       </c>
     </row>
@@ -984,7 +1191,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>&gt;= 60.0% + Trend Guard H1</t>
+          <t>Technical Confluence (Stoch RSI + Patterns v3.4)</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1215,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>5 Trade</t>
+          <t>8 Trade</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1227,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>8.0%</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1239,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>3 Trade</t>
+          <t>5 Trade</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1251,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2 Trade</t>
+          <t>3 Trade</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1263,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>60.00%</t>
+          <t>62.50%</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1275,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>$+15.51 USD</t>
+          <t>$+15.20 USD</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1287,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>$+3.10 USD</t>
+          <t>$+1.90 USD</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1299,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>2.88</t>
+          <t>2.35</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1311,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10 02:09:27 WIB</t>
+          <t>2026-09-11 17:08:27 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>